<commit_message>
Delivery log: add R-004, R-006; correct R-008
</commit_message>
<xml_diff>
--- a/static/case-study/downloads/implementation-delivery-log.xlsx
+++ b/static/case-study/downloads/implementation-delivery-log.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcdel\Root\01_PROJECTS\06_job_applications\BA_BPMN\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcdel\Root\01_PROJECTS\qld-traffic-monitor\static\case-study\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237C2BFC-D3A5-4E17-9E14-FB73A5F643EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9933687D-16C1-4282-87BF-44F778427607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>Requirement</t>
   </si>
@@ -102,16 +102,37 @@
     <t>R-008</t>
   </si>
   <si>
-    <t>Collection completeness</t>
-  </si>
-  <si>
-    <t>Record collection status/failures</t>
-  </si>
-  <si>
-    <t>Logs / monitoring evidence</t>
-  </si>
-  <si>
     <t>https://traffic.jcdelgado.dev</t>
+  </si>
+  <si>
+    <t>Snapshot export and analysis notebook</t>
+  </si>
+  <si>
+    <t>Export the database to CSV, analyse it in Python and publish the results as a report</t>
+  </si>
+  <si>
+    <t>https://traffic.jcdelgado.dev/report</t>
+  </si>
+  <si>
+    <t>R-004</t>
+  </si>
+  <si>
+    <t>Time since latest crash</t>
+  </si>
+  <si>
+    <t>Show the latest crash's start time in Brisbane time and the time elapsed since</t>
+  </si>
+  <si>
+    <t>R-006</t>
+  </si>
+  <si>
+    <t>Not implemented</t>
+  </si>
+  <si>
+    <t>Deferred: low value relative to effort at project close. The worker logs failed polls and retries, but nothing is stored</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
 </sst>
 </file>
@@ -164,7 +185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -175,12 +196,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -200,21 +239,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -229,13 +253,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{97BAF26A-1509-4324-9F11-0E4A80A58490}" name="Table1" displayName="Table1" ref="A1:D9" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:D9" xr:uid="{97BAF26A-1509-4324-9F11-0E4A80A58490}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{97BAF26A-1509-4324-9F11-0E4A80A58490}" name="Table1" displayName="Table1" ref="A1:D11" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:D11" xr:uid="{97BAF26A-1509-4324-9F11-0E4A80A58490}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{7912AECF-583D-4F7A-88C9-D43D2C4CC2FD}" name="Requirement" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{1126E72E-9554-4348-998B-8AA4E6DD40AC}" name="What was delivered" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{CF954643-7014-406F-B722-39BD9C61081D}" name="Implementation decision" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{F7951C88-46AA-456F-ADC9-B5A14722F6B5}" name="Evidence" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{7912AECF-583D-4F7A-88C9-D43D2C4CC2FD}" name="Requirement" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{1126E72E-9554-4348-998B-8AA4E6DD40AC}" name="What was delivered" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{CF954643-7014-406F-B722-39BD9C61081D}" name="Implementation decision" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{F7951C88-46AA-456F-ADC9-B5A14722F6B5}" name="Evidence" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -504,13 +528,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.77734375" customWidth="1"/>
     <col min="2" max="2" width="19.33203125" customWidth="1"/>
     <col min="3" max="3" width="23.77734375" customWidth="1"/>
-    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -569,67 +593,97 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+    <row r="9" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+      <c r="B9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D5" r:id="rId1" xr:uid="{9356C041-1D4F-4722-B6C4-5A1820A24D2C}"/>
+    <hyperlink ref="D6" r:id="rId1" xr:uid="{9356C041-1D4F-4722-B6C4-5A1820A24D2C}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{1D7B8318-837D-44AB-A33B-9F4987EAC67B}"/>
+    <hyperlink ref="D7" r:id="rId3" display="https://traffic.jcdelgado.dev/" xr:uid="{FCB8982F-56CD-4583-A386-988F8D7697CB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>